<commit_message>
image links update v2
</commit_message>
<xml_diff>
--- a/radioaparat_linkovi.xlsx
+++ b/radioaparat_linkovi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/m1l0s/Library/Mobile Documents/com~apple~CloudDocs/Apple/iOS apps/radioAPARAT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475AB8BD-A8D4-F545-A62A-903FBECA59A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D7E438-7452-A449-95FF-5B6EEC6F8A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16880" xr2:uid="{6FF80182-A761-2647-9A5D-CE1327C51E42}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="254">
   <si>
     <t>ID</t>
   </si>
@@ -592,10 +592,6 @@
   </si>
   <si>
     <t>utorkom od 18.00 do 20.00</t>
-  </si>
-  <si>
-    <t>Ovim programom knjižara Beopolis proširuje komunikaciju sa publikom, obrađujući teme iz kulture, književnosti, obrazovanja, politike i sporta.
-Emisiju uređuje i vodi: Aleksandar (Kafka) Nikolić, osnivač Beopolisa</t>
   </si>
   <si>
     <t>svakog poslednjeg ponedeljka u mesecu od 17 do 18h</t>
@@ -786,6 +782,68 @@
   </si>
   <si>
     <t>https://radioaparat.rs/h-content/uploads/2022/01/Preslicavanje-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/podzemlje-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/mono-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/03/mansarda-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/dirizabl-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/ekspedicija-radio-aparat.png</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/orfejeva-kutija-radio-aparat-1200x762.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/reality-check-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/beopolis-iz-radio-aparata-radio-aparat-1200x525.jpg</t>
+  </si>
+  <si>
+    <t>Beopolis je kultna beogradska knjižara osnovana krajem 1999. godine, u saradnji sa Domom omladine Begrada. Uprkos izazovima i teškim periodima, knjižara je opstala i danas je mesto koje ima značajnu društvenu i kulturnu ulogu u Beogradu, Srbiji i regionu bivše Jugoslavije. Ključni programi Beopolisa obuhvataju pažljivu selekciju nekomercijalne i komercijalne književnosti, promociju relevantnih naslova iz oblasti humanistike, umetnosti, stripa i regionalne književnosti. Beopolis programski pruža podršku nezavisnim i malim izdavačima, učestvuje u organizovanju književnih promocija, tribina, diskusija, festivala. Prepoznat kao prostor okrenut alternativnom i kritičkom, odnos Beopolisa i zajednice je izrazito interaktivan i zasnovan na uzajamnom poverenju. Beopolis je svojim angažmanom i ponekad čak subverzirvnim stavom prema rigidnim i zatvorenim umetničkim i društvenim politikama i praksama, stvorio generacije angažovanih čitalaca i podsticao otvorene diskusije o važnim društvenim i kulturnim pitanjima kroz promociju umetničkih i svih drugih sloboda.
+Knjižara Beopolis od 2016. godine sarađuje sa RadioAparatom. Emisija „Beopolis iz RadioAparata“ emituje se utorkom od 18 do 20 časova i ovim programom knjižara proširuje komunikaciju sa publikom, obrađujući teme iz kulture, književnosti, obrazovanja, politike i sporta. Ova saradnja omogućava Beopolisu da svoje ideje i stavove komunicira putem savremenih medija, jačajući svoju povezanost sa lokalnom i regionalnom zajednicom.
+Emisiju uređuje i vodi Aleksandar (Kafka) Nikolić, osnivač Beopolisa</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/grad-u-prolazu-radio-aparat-1200x800.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/kamilica-radio-aparat.png</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/03/kultur-kajgana-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/sceniranje-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/antroposestvije-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/Liceulice-FM-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/Radio-galaksija-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2025/09/Sizoanaliza-radio-aparat-1200x1200.png</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/Nevergrin-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/Pop-Kujna-radio-aparat.jpg</t>
+  </si>
+  <si>
+    <t>https://radioaparat.rs/h-content/uploads/2022/01/povratak-lopova-radio-aparat-1200x675.png</t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1238,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC0F6B4F-BD8C-3745-9181-6C92BF1467A2}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:M57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1251,7 +1308,7 @@
         <v>122</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1271,7 +1328,7 @@
         <v>140</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>126</v>
@@ -1280,7 +1337,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1308,7 +1365,7 @@
         <v>128</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1322,10 +1379,13 @@
         <v>11</v>
       </c>
       <c r="D6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>209</v>
+      <c r="F6" s="3" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1344,8 +1404,11 @@
       <c r="E7" s="6" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F7" s="3" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1372,6 +1435,9 @@
       <c r="E9" s="6" t="s">
         <v>156</v>
       </c>
+      <c r="F9" s="3" t="s">
+        <v>236</v>
+      </c>
       <c r="H9" s="4" t="s">
         <v>159</v>
       </c>
@@ -1399,10 +1465,10 @@
         <v>148</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>227</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>150</v>
@@ -1411,7 +1477,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -1433,16 +1499,19 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="K12" s="4" t="s">
         <v>211</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1461,6 +1530,9 @@
       <c r="E13" s="6" t="s">
         <v>130</v>
       </c>
+      <c r="F13" s="3" t="s">
+        <v>238</v>
+      </c>
       <c r="I13" s="4" t="s">
         <v>131</v>
       </c>
@@ -1482,13 +1554,13 @@
         <v>142</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -1499,7 +1571,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -1530,7 +1602,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -1541,7 +1613,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -1563,13 +1635,13 @@
         <v>11</v>
       </c>
       <c r="D20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -1580,7 +1652,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1602,13 +1674,13 @@
         <v>11</v>
       </c>
       <c r="D23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="E23" s="6" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -1630,10 +1702,10 @@
         <v>11</v>
       </c>
       <c r="D25" t="s">
+        <v>216</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>217</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="26" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1647,10 +1719,13 @@
         <v>11</v>
       </c>
       <c r="D26" t="s">
+        <v>218</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="E26" s="6" t="s">
-        <v>220</v>
+      <c r="F26" s="3" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="27" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1670,7 +1745,7 @@
         <v>139</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>143</v>
@@ -1699,7 +1774,7 @@
         <v>147</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1713,13 +1788,13 @@
         <v>11</v>
       </c>
       <c r="D29" t="s">
+        <v>220</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="E29" s="6" t="s">
-        <v>222</v>
-      </c>
       <c r="F29" s="3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1738,6 +1813,9 @@
       <c r="E30" s="6" t="s">
         <v>152</v>
       </c>
+      <c r="F30" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="K30" s="4" t="s">
         <v>154</v>
       </c>
@@ -1745,7 +1823,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -1770,7 +1848,10 @@
         <v>178</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>179</v>
+        <v>242</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1789,8 +1870,11 @@
       <c r="E33" s="6" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F33" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>19</v>
       </c>
@@ -1817,6 +1901,9 @@
       <c r="E35" s="6" t="s">
         <v>169</v>
       </c>
+      <c r="F35" s="3" t="s">
+        <v>244</v>
+      </c>
       <c r="H35" s="4" t="s">
         <v>170</v>
       </c>
@@ -1838,13 +1925,16 @@
         <v>20</v>
       </c>
       <c r="D36" t="s">
+        <v>222</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="E36" s="6" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F36" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>85</v>
       </c>
@@ -1871,6 +1961,9 @@
       <c r="E38" s="6" t="s">
         <v>174</v>
       </c>
+      <c r="F38" s="3" t="s">
+        <v>246</v>
+      </c>
       <c r="H38" s="4" t="s">
         <v>177</v>
       </c>
@@ -1881,7 +1974,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>86</v>
       </c>
@@ -1892,7 +1985,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="40" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>87</v>
       </c>
@@ -1903,7 +1996,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>89</v>
       </c>
@@ -1914,7 +2007,7 @@
         <v>24</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1928,13 +2021,16 @@
         <v>24</v>
       </c>
       <c r="D42" t="s">
+        <v>179</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F42" s="3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>93</v>
       </c>
@@ -1945,10 +2041,10 @@
         <v>24</v>
       </c>
       <c r="E43" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="K43" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="K43" s="4" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -1967,6 +2063,9 @@
       <c r="E44" s="6" t="s">
         <v>163</v>
       </c>
+      <c r="F44" s="3" t="s">
+        <v>248</v>
+      </c>
       <c r="H44" s="4" t="s">
         <v>164</v>
       </c>
@@ -1985,10 +2084,13 @@
         <v>24</v>
       </c>
       <c r="D45" t="s">
+        <v>183</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="E45" s="6" t="s">
-        <v>185</v>
+      <c r="F45" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2002,16 +2104,19 @@
         <v>24</v>
       </c>
       <c r="D46" t="s">
+        <v>185</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="F46" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="J46" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="J46" s="4" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>100</v>
       </c>
@@ -2022,19 +2127,19 @@
         <v>24</v>
       </c>
       <c r="E47" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K47" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="H47" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="K47" s="4" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>23</v>
       </c>
@@ -2045,7 +2150,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>103</v>
       </c>
@@ -2067,10 +2172,10 @@
         <v>107</v>
       </c>
       <c r="D50" t="s">
+        <v>192</v>
+      </c>
+      <c r="E50" s="6" t="s">
         <v>193</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2084,10 +2189,13 @@
         <v>107</v>
       </c>
       <c r="D51" t="s">
+        <v>194</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="E51" s="6" t="s">
-        <v>196</v>
+      <c r="F51" s="3" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2101,13 +2209,16 @@
         <v>107</v>
       </c>
       <c r="D52" t="s">
+        <v>196</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="F52" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="K52" s="4" t="s">
         <v>198</v>
-      </c>
-      <c r="K52" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="53" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2121,10 +2232,13 @@
         <v>107</v>
       </c>
       <c r="D53" t="s">
+        <v>199</v>
+      </c>
+      <c r="E53" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="E53" s="6" t="s">
-        <v>201</v>
+      <c r="F53" s="3" t="s">
+        <v>253</v>
       </c>
     </row>
     <row r="54" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2138,10 +2252,10 @@
         <v>107</v>
       </c>
       <c r="D54" t="s">
+        <v>201</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>202</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="55" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2155,10 +2269,10 @@
         <v>107</v>
       </c>
       <c r="D55" t="s">
+        <v>203</v>
+      </c>
+      <c r="E55" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="56" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -2172,13 +2286,13 @@
         <v>107</v>
       </c>
       <c r="D56" t="s">
+        <v>205</v>
+      </c>
+      <c r="E56" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="E56" s="6" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="16" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>118</v>
       </c>
@@ -2190,13 +2304,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M57" xr:uid="{CC0F6B4F-BD8C-3745-9181-6C92BF1467A2}">
-    <filterColumn colId="3">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M57" xr:uid="{CC0F6B4F-BD8C-3745-9181-6C92BF1467A2}"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -2246,6 +2354,25 @@
     <hyperlink ref="F27" r:id="rId38" xr:uid="{D6FDBEA1-7B6C-8B42-8C9E-B7CA7ABAB517}"/>
     <hyperlink ref="F28" r:id="rId39" xr:uid="{C09773AE-599C-EB45-9BCA-089076AC6614}"/>
     <hyperlink ref="F29" r:id="rId40" xr:uid="{F0534A1E-B569-654F-82FE-2F90A0010A96}"/>
+    <hyperlink ref="F6" r:id="rId41" xr:uid="{30F7D488-149B-6D49-B919-800B2A68C852}"/>
+    <hyperlink ref="F7" r:id="rId42" xr:uid="{B0F0E3C0-8526-0740-B889-6BF3422E60D3}"/>
+    <hyperlink ref="F9" r:id="rId43" xr:uid="{970E7787-AD1F-2B4D-B08C-B58ACF970A3E}"/>
+    <hyperlink ref="F12" r:id="rId44" xr:uid="{24441B47-EA18-E04D-B8EF-CA177C9A9AC4}"/>
+    <hyperlink ref="F13" r:id="rId45" xr:uid="{781FE32F-D880-C64D-A04E-D7A460986DCD}"/>
+    <hyperlink ref="F26" r:id="rId46" xr:uid="{193D7892-2EEF-6141-97F2-3D708C3D2CC1}"/>
+    <hyperlink ref="F30" r:id="rId47" xr:uid="{09797570-22FA-A141-BD6D-10F41D09BB0D}"/>
+    <hyperlink ref="F32" r:id="rId48" xr:uid="{F0934C9E-58EE-FF4B-B8A9-786637D5EEBE}"/>
+    <hyperlink ref="F33" r:id="rId49" xr:uid="{CA91CB82-3F3D-FF45-A67F-6454E70D288C}"/>
+    <hyperlink ref="F35" r:id="rId50" xr:uid="{6A3BE2F8-D9B0-D542-9F53-79DB2B7BD564}"/>
+    <hyperlink ref="F36" r:id="rId51" xr:uid="{90778B8B-230E-3C4E-BB69-AB5EF45FC911}"/>
+    <hyperlink ref="F38" r:id="rId52" xr:uid="{1BA9A77C-4A85-F24E-8AF9-B50B5AFB6E33}"/>
+    <hyperlink ref="F42" r:id="rId53" xr:uid="{FEB38D6B-D4E6-7B45-99E8-4E3C90DB13B2}"/>
+    <hyperlink ref="F44" r:id="rId54" xr:uid="{33DB0183-6916-324A-AD18-7C1452F8C73C}"/>
+    <hyperlink ref="F45" r:id="rId55" xr:uid="{26B7D58B-9311-0C4B-B099-7065EDCA4718}"/>
+    <hyperlink ref="F46" r:id="rId56" xr:uid="{EE61F8FE-7073-FE4D-8099-1E981028660D}"/>
+    <hyperlink ref="F51" r:id="rId57" xr:uid="{E44A0830-EE46-AF4E-8BB7-2EF2807ABD62}"/>
+    <hyperlink ref="F52" r:id="rId58" xr:uid="{58FC44C0-BBDF-D144-B565-0B23179055B8}"/>
+    <hyperlink ref="F53" r:id="rId59" xr:uid="{944162AC-BD30-0E4F-9B64-E4E37111A29A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>